<commit_message>
add llama3.1 70B and 8B RAG results and scripts
</commit_message>
<xml_diff>
--- a/rag/eval/results_full150/SuppFile2_Stats_generated.xlsx
+++ b/rag/eval/results_full150/SuppFile2_Stats_generated.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IndividQuest_FisherExact(Tab3)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelComp_SignedRankFig4" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelComp_BH_AdjustFig4" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="IndividQuest_FisherExact(Tab3)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ModelComp_SignedRankFig4" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ModelComp_BH_AdjustFig4" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -707,7 +707,7 @@
         <v>7</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.157</v>
+        <v>0.214</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         <v>9</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.919</v>
+        <v>0.798</v>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
@@ -735,7 +735,7 @@
         <v>8</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.153</v>
+        <v>0.133</v>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         <v>1</v>
       </c>
       <c r="Z3" s="3" t="n">
-        <v>0.000319</v>
+        <v>0.000217</v>
       </c>
       <c r="AA3" s="3" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         <v>1</v>
       </c>
       <c r="AE3" s="3" t="n">
-        <v>0.00513</v>
+        <v>0.00291</v>
       </c>
       <c r="AF3" s="3" t="inlineStr">
         <is>
@@ -853,7 +853,7 @@
         <v>10</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         <v>7</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.676</v>
+        <v>0.738</v>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
@@ -1288,15 +1288,15 @@
       <c r="X7" t="n">
         <v>0.0066</v>
       </c>
-      <c r="Y7" s="4" t="n">
+      <c r="Y7" t="n">
         <v>5</v>
       </c>
-      <c r="Z7" s="4" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="AA7" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="Z7" t="n">
+        <v>0.0587</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AC7" t="n">
@@ -1320,7 +1320,7 @@
         <v>1</v>
       </c>
       <c r="AJ7" s="3" t="n">
-        <v>0.000597</v>
+        <v>0.0005419999999999999</v>
       </c>
       <c r="AK7" s="3" t="inlineStr">
         <is>
@@ -1410,7 +1410,7 @@
         <v>6</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.501</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
         <v>4</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.031</v>
+        <v>0.0302</v>
       </c>
       <c r="AK8" s="4" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
         <v>8</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.446</v>
+        <v>0.608</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
         <v>5</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.913</v>
+        <v>0.9</v>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
         <v>6</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.213</v>
+        <v>0.291</v>
       </c>
       <c r="AK10" t="inlineStr">
         <is>
@@ -1754,7 +1754,7 @@
         <v>11</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.879</v>
+        <v>0.85</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -1782,7 +1782,7 @@
         <v>11</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.759</v>
+        <v>0.862</v>
       </c>
       <c r="AK11" t="inlineStr">
         <is>
@@ -1872,7 +1872,7 @@
         <v>4</v>
       </c>
       <c r="Z12" s="4" t="n">
-        <v>0.0293</v>
+        <v>0.0266</v>
       </c>
       <c r="AA12" s="4" t="inlineStr">
         <is>
@@ -1886,7 +1886,7 @@
         <v>8</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.702</v>
+        <v>0.662</v>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
@@ -1900,7 +1900,7 @@
         <v>2</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.0107</v>
+        <v>0.0146</v>
       </c>
       <c r="AK12" s="4" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
         <v>10</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.992</v>
+        <v>1</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
         <v>6</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.462</v>
+        <v>0.438</v>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
@@ -2018,7 +2018,7 @@
         <v>7</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.138</v>
+        <v>0.104</v>
       </c>
       <c r="AK13" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         <v>9</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.701</v>
+        <v>0.864</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -2235,7 +2235,7 @@
         <v>4</v>
       </c>
       <c r="AE15" t="n">
-        <v>0.226</v>
+        <v>0.277</v>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
@@ -2249,7 +2249,7 @@
         <v>5</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.0594</v>
+        <v>0.054</v>
       </c>
       <c r="AK15" t="inlineStr">
         <is>
@@ -2334,7 +2334,7 @@
         <v>2</v>
       </c>
       <c r="Z16" s="3" t="n">
-        <v>0.00292</v>
+        <v>0.00398</v>
       </c>
       <c r="AA16" s="3" t="inlineStr">
         <is>
@@ -2344,13 +2344,13 @@
       <c r="AC16" t="n">
         <v>0.00361</v>
       </c>
-      <c r="AD16" s="3" t="n">
+      <c r="AD16" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="AE16" s="3" t="n">
-        <v>0.00993</v>
-      </c>
-      <c r="AF16" s="3" t="inlineStr">
+      <c r="AE16" s="4" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="AF16" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -2362,7 +2362,7 @@
         <v>9</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0.301</v>
+        <v>0.274</v>
       </c>
       <c r="AK16" t="inlineStr">
         <is>
@@ -2447,7 +2447,7 @@
         <v>3</v>
       </c>
       <c r="Z17" s="3" t="n">
-        <v>0.00178</v>
+        <v>0.00243</v>
       </c>
       <c r="AA17" s="3" t="inlineStr">
         <is>
@@ -2461,7 +2461,7 @@
         <v>3</v>
       </c>
       <c r="AE17" s="4" t="n">
-        <v>0.0175</v>
+        <v>0.0239</v>
       </c>
       <c r="AF17" s="4" t="inlineStr">
         <is>
@@ -2471,15 +2471,15 @@
       <c r="AH17" t="n">
         <v>0.0138</v>
       </c>
-      <c r="AI17" t="n">
+      <c r="AI17" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="AJ17" t="n">
-        <v>0.0506</v>
-      </c>
-      <c r="AK17" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="AJ17" s="4" t="n">
+        <v>0.0414</v>
+      </c>
+      <c r="AK17" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
         <v>10</v>
       </c>
       <c r="AE19" t="n">
-        <v>0.919</v>
+        <v>0.798</v>
       </c>
       <c r="AF19" t="inlineStr">
         <is>
@@ -2589,7 +2589,7 @@
         <v>5</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0.203</v>
+        <v>0.192</v>
       </c>
       <c r="AK19" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         <v>3</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.295</v>
+        <v>0.287</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -2688,7 +2688,7 @@
         <v>7</v>
       </c>
       <c r="AE20" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.528</v>
       </c>
       <c r="AF20" t="inlineStr">
         <is>
@@ -2787,7 +2787,7 @@
         <v>4</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.755</v>
+        <v>0.735</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -2801,7 +2801,7 @@
         <v>4</v>
       </c>
       <c r="AE21" t="n">
-        <v>0.365</v>
+        <v>0.356</v>
       </c>
       <c r="AF21" t="inlineStr">
         <is>
@@ -3027,7 +3027,7 @@
         <v>11</v>
       </c>
       <c r="AE23" t="n">
-        <v>0.915</v>
+        <v>0.749</v>
       </c>
       <c r="AF23" t="inlineStr">
         <is>
@@ -3041,7 +3041,7 @@
         <v>10</v>
       </c>
       <c r="AJ23" t="n">
-        <v>0.981</v>
+        <v>1</v>
       </c>
       <c r="AK23" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
         <v>5</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.49</v>
+        <v>0.547</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -3140,7 +3140,7 @@
         <v>1</v>
       </c>
       <c r="AE24" s="4" t="n">
-        <v>0.0133</v>
+        <v>0.0129</v>
       </c>
       <c r="AF24" s="4" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
         <v>1</v>
       </c>
       <c r="AJ24" s="3" t="n">
-        <v>0.000128</v>
+        <v>8.7e-05</v>
       </c>
       <c r="AK24" s="3" t="inlineStr">
         <is>
@@ -3239,7 +3239,7 @@
         <v>9</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.822</v>
+        <v>1</v>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
@@ -3253,7 +3253,7 @@
         <v>2</v>
       </c>
       <c r="AE25" t="n">
-        <v>0.08210000000000001</v>
+        <v>0.0799</v>
       </c>
       <c r="AF25" t="inlineStr">
         <is>
@@ -3267,7 +3267,7 @@
         <v>2</v>
       </c>
       <c r="AJ25" s="3" t="n">
-        <v>0.00847</v>
+        <v>0.00693</v>
       </c>
       <c r="AK25" s="3" t="inlineStr">
         <is>
@@ -3352,7 +3352,7 @@
         <v>2</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.544</v>
+        <v>0.495</v>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
         <v>3</v>
       </c>
       <c r="AE26" t="n">
-        <v>0.506</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AF26" t="inlineStr">
         <is>
@@ -3465,7 +3465,7 @@
         <v>8</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.665</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="AA27" t="inlineStr">
         <is>
@@ -3479,7 +3479,7 @@
         <v>12</v>
       </c>
       <c r="AE27" t="n">
-        <v>0.913</v>
+        <v>0.9</v>
       </c>
       <c r="AF27" t="inlineStr">
         <is>
@@ -3493,7 +3493,7 @@
         <v>8</v>
       </c>
       <c r="AJ27" t="n">
-        <v>0.487</v>
+        <v>0.59</v>
       </c>
       <c r="AK27" t="inlineStr">
         <is>
@@ -3592,7 +3592,7 @@
         <v>13</v>
       </c>
       <c r="AE28" t="n">
-        <v>1</v>
+        <v>0.979</v>
       </c>
       <c r="AF28" t="inlineStr">
         <is>
@@ -3691,7 +3691,7 @@
         <v>1</v>
       </c>
       <c r="Z29" t="n">
-        <v>0.292</v>
+        <v>0.254</v>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
@@ -3719,7 +3719,7 @@
         <v>3</v>
       </c>
       <c r="AJ29" t="n">
-        <v>0.111</v>
+        <v>0.152</v>
       </c>
       <c r="AK29" t="inlineStr">
         <is>
@@ -3804,7 +3804,7 @@
         <v>6</v>
       </c>
       <c r="Z30" t="n">
-        <v>0.988</v>
+        <v>1</v>
       </c>
       <c r="AA30" t="inlineStr">
         <is>
@@ -3818,7 +3818,7 @@
         <v>6</v>
       </c>
       <c r="AE30" t="n">
-        <v>0.536</v>
+        <v>0.522</v>
       </c>
       <c r="AF30" t="inlineStr">
         <is>
@@ -3832,7 +3832,7 @@
         <v>4</v>
       </c>
       <c r="AJ30" t="n">
-        <v>0.202</v>
+        <v>0.165</v>
       </c>
       <c r="AK30" t="inlineStr">
         <is>
@@ -3931,7 +3931,7 @@
         <v>9</v>
       </c>
       <c r="AE31" t="n">
-        <v>1</v>
+        <v>0.898</v>
       </c>
       <c r="AF31" t="inlineStr">
         <is>
@@ -4044,7 +4044,7 @@
         <v>5</v>
       </c>
       <c r="AE32" t="n">
-        <v>0.312</v>
+        <v>0.387</v>
       </c>
       <c r="AF32" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
         <v>9</v>
       </c>
       <c r="AJ32" t="n">
-        <v>0.492</v>
+        <v>0.509</v>
       </c>
       <c r="AK32" t="inlineStr">
         <is>
@@ -4143,7 +4143,7 @@
         <v>10</v>
       </c>
       <c r="Z33" t="n">
-        <v>0.881</v>
+        <v>0.858</v>
       </c>
       <c r="AA33" t="inlineStr">
         <is>
@@ -4157,7 +4157,7 @@
         <v>8</v>
       </c>
       <c r="AE33" t="n">
-        <v>0.512</v>
+        <v>0.537</v>
       </c>
       <c r="AF33" t="inlineStr">
         <is>
@@ -4171,7 +4171,7 @@
         <v>7</v>
       </c>
       <c r="AJ33" t="n">
-        <v>0.332</v>
+        <v>0.314</v>
       </c>
       <c r="AK33" t="inlineStr">
         <is>
@@ -4284,7 +4284,7 @@
         <v>6</v>
       </c>
       <c r="AJ34" t="n">
-        <v>0.273</v>
+        <v>0.29</v>
       </c>
       <c r="AK34" t="inlineStr">
         <is>
@@ -4371,7 +4371,7 @@
         <v>6</v>
       </c>
       <c r="Z37" t="n">
-        <v>0.389</v>
+        <v>0.477</v>
       </c>
       <c r="AA37" t="inlineStr">
         <is>
@@ -4399,7 +4399,7 @@
         <v>6</v>
       </c>
       <c r="AJ37" t="n">
-        <v>0.265</v>
+        <v>0.258</v>
       </c>
       <c r="AK37" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
         <v>10</v>
       </c>
       <c r="AE38" t="n">
-        <v>0.575</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AF38" t="inlineStr">
         <is>
@@ -4512,7 +4512,7 @@
         <v>5</v>
       </c>
       <c r="AJ38" t="n">
-        <v>0.519</v>
+        <v>0.708</v>
       </c>
       <c r="AK38" t="inlineStr">
         <is>
@@ -4597,7 +4597,7 @@
         <v>7</v>
       </c>
       <c r="Z39" t="n">
-        <v>0.895</v>
+        <v>0.915</v>
       </c>
       <c r="AA39" t="inlineStr">
         <is>
@@ -4611,7 +4611,7 @@
         <v>5</v>
       </c>
       <c r="AE39" t="n">
-        <v>0.171</v>
+        <v>0.234</v>
       </c>
       <c r="AF39" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         <v>4</v>
       </c>
       <c r="AJ39" t="n">
-        <v>0.555</v>
+        <v>0.758</v>
       </c>
       <c r="AK39" t="inlineStr">
         <is>
@@ -4837,7 +4837,7 @@
         <v>8</v>
       </c>
       <c r="AE41" t="n">
-        <v>0.543</v>
+        <v>0.412</v>
       </c>
       <c r="AF41" t="inlineStr">
         <is>
@@ -4851,7 +4851,7 @@
         <v>9</v>
       </c>
       <c r="AJ41" t="n">
-        <v>0.981</v>
+        <v>1</v>
       </c>
       <c r="AK41" t="inlineStr">
         <is>
@@ -4936,7 +4936,7 @@
         <v>4</v>
       </c>
       <c r="Z42" t="n">
-        <v>0.359</v>
+        <v>0.408</v>
       </c>
       <c r="AA42" t="inlineStr">
         <is>
@@ -4950,7 +4950,7 @@
         <v>6</v>
       </c>
       <c r="AE42" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="AF42" t="inlineStr">
         <is>
@@ -4964,7 +4964,7 @@
         <v>12</v>
       </c>
       <c r="AJ42" t="n">
-        <v>0.727</v>
+        <v>0.779</v>
       </c>
       <c r="AK42" t="inlineStr">
         <is>
@@ -5049,7 +5049,7 @@
         <v>11</v>
       </c>
       <c r="Z43" t="n">
-        <v>0.822</v>
+        <v>1</v>
       </c>
       <c r="AA43" t="inlineStr">
         <is>
@@ -5063,7 +5063,7 @@
         <v>9</v>
       </c>
       <c r="AE43" t="n">
-        <v>0.37</v>
+        <v>0.404</v>
       </c>
       <c r="AF43" t="inlineStr">
         <is>
@@ -5176,7 +5176,7 @@
         <v>11</v>
       </c>
       <c r="AE44" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="AF44" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
         <v>10</v>
       </c>
       <c r="Z45" t="n">
-        <v>0.778</v>
+        <v>0.891</v>
       </c>
       <c r="AA45" t="inlineStr">
         <is>
@@ -5289,7 +5289,7 @@
         <v>13</v>
       </c>
       <c r="AE45" t="n">
-        <v>0.913</v>
+        <v>0.9</v>
       </c>
       <c r="AF45" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
         <v>14</v>
       </c>
       <c r="AJ45" t="n">
-        <v>0.985</v>
+        <v>1</v>
       </c>
       <c r="AK45" t="inlineStr">
         <is>
@@ -5388,7 +5388,7 @@
         <v>5</v>
       </c>
       <c r="Z46" t="n">
-        <v>0.323</v>
+        <v>0.33</v>
       </c>
       <c r="AA46" t="inlineStr">
         <is>
@@ -5416,7 +5416,7 @@
         <v>3</v>
       </c>
       <c r="AJ46" t="n">
-        <v>0.187</v>
+        <v>0.255</v>
       </c>
       <c r="AK46" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
         <v>4</v>
       </c>
       <c r="AE47" t="n">
-        <v>0.104</v>
+        <v>0.0945</v>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
@@ -5529,7 +5529,7 @@
         <v>8</v>
       </c>
       <c r="AJ47" t="n">
-        <v>0.701</v>
+        <v>0.715</v>
       </c>
       <c r="AK47" t="inlineStr">
         <is>
@@ -5628,7 +5628,7 @@
         <v>7</v>
       </c>
       <c r="AE48" t="n">
-        <v>0.227</v>
+        <v>0.232</v>
       </c>
       <c r="AF48" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
         <v>10</v>
       </c>
       <c r="AJ48" t="n">
-        <v>0.781</v>
+        <v>0.71</v>
       </c>
       <c r="AK48" t="inlineStr">
         <is>
@@ -5741,7 +5741,7 @@
         <v>12</v>
       </c>
       <c r="AE49" t="n">
-        <v>1</v>
+        <v>0.919</v>
       </c>
       <c r="AF49" t="inlineStr">
         <is>
@@ -5840,7 +5840,7 @@
         <v>3</v>
       </c>
       <c r="Z50" t="n">
-        <v>0.297</v>
+        <v>0.405</v>
       </c>
       <c r="AA50" t="inlineStr">
         <is>
@@ -5854,7 +5854,7 @@
         <v>1</v>
       </c>
       <c r="AE50" s="3" t="n">
-        <v>0.00147</v>
+        <v>0.002</v>
       </c>
       <c r="AF50" s="3" t="inlineStr">
         <is>
@@ -5868,7 +5868,7 @@
         <v>7</v>
       </c>
       <c r="AJ50" t="n">
-        <v>0.492</v>
+        <v>0.516</v>
       </c>
       <c r="AK50" t="inlineStr">
         <is>
@@ -5953,7 +5953,7 @@
         <v>2</v>
       </c>
       <c r="Z51" s="3" t="n">
-        <v>0.00117</v>
+        <v>0.00159</v>
       </c>
       <c r="AA51" s="3" t="inlineStr">
         <is>
@@ -5967,7 +5967,7 @@
         <v>2</v>
       </c>
       <c r="AE51" s="3" t="n">
-        <v>0.00196</v>
+        <v>0.00267</v>
       </c>
       <c r="AF51" s="3" t="inlineStr">
         <is>
@@ -5981,7 +5981,7 @@
         <v>1</v>
       </c>
       <c r="AJ51" s="3" t="n">
-        <v>0.00151</v>
+        <v>0.00103</v>
       </c>
       <c r="AK51" s="3" t="inlineStr">
         <is>
@@ -6066,7 +6066,7 @@
         <v>1</v>
       </c>
       <c r="Z52" s="3" t="n">
-        <v>1.47e-05</v>
+        <v>2e-05</v>
       </c>
       <c r="AA52" s="3" t="inlineStr">
         <is>
@@ -6080,7 +6080,7 @@
         <v>3</v>
       </c>
       <c r="AE52" s="3" t="n">
-        <v>0.00429</v>
+        <v>0.00585</v>
       </c>
       <c r="AF52" s="3" t="inlineStr">
         <is>
@@ -6094,7 +6094,7 @@
         <v>2</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>0.0455</v>
+        <v>0.031</v>
       </c>
       <c r="AK52" s="4" t="inlineStr">
         <is>
@@ -6180,7 +6180,7 @@
         <v>5</v>
       </c>
       <c r="Z54" t="n">
-        <v>0.0591</v>
+        <v>0.0806</v>
       </c>
       <c r="AA54" t="inlineStr">
         <is>
@@ -6194,7 +6194,7 @@
         <v>11</v>
       </c>
       <c r="AE54" t="n">
-        <v>0.983</v>
+        <v>0.928</v>
       </c>
       <c r="AF54" t="inlineStr">
         <is>
@@ -6208,7 +6208,7 @@
         <v>1</v>
       </c>
       <c r="AJ54" s="3" t="n">
-        <v>0.000574</v>
+        <v>0.000559</v>
       </c>
       <c r="AK54" s="3" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         <v>3</v>
       </c>
       <c r="Z55" s="3" t="n">
-        <v>0.00297</v>
+        <v>0.0027</v>
       </c>
       <c r="AA55" s="3" t="inlineStr">
         <is>
@@ -6307,7 +6307,7 @@
         <v>3</v>
       </c>
       <c r="AE55" s="4" t="n">
-        <v>0.0334</v>
+        <v>0.0285</v>
       </c>
       <c r="AF55" s="4" t="inlineStr">
         <is>
@@ -6406,7 +6406,7 @@
         <v>11</v>
       </c>
       <c r="Z56" t="n">
-        <v>0.755</v>
+        <v>0.735</v>
       </c>
       <c r="AA56" t="inlineStr">
         <is>
@@ -6420,7 +6420,7 @@
         <v>7</v>
       </c>
       <c r="AE56" t="n">
-        <v>0.635</v>
+        <v>0.673</v>
       </c>
       <c r="AF56" t="inlineStr">
         <is>
@@ -6519,7 +6519,7 @@
         <v>12</v>
       </c>
       <c r="Z57" t="n">
-        <v>0.913</v>
+        <v>1</v>
       </c>
       <c r="AA57" t="inlineStr">
         <is>
@@ -6632,7 +6632,7 @@
         <v>13</v>
       </c>
       <c r="Z58" t="n">
-        <v>1</v>
+        <v>0.898</v>
       </c>
       <c r="AA58" t="inlineStr">
         <is>
@@ -6660,7 +6660,7 @@
         <v>11</v>
       </c>
       <c r="AJ58" t="n">
-        <v>0.981</v>
+        <v>1</v>
       </c>
       <c r="AK58" t="inlineStr">
         <is>
@@ -6741,15 +6741,15 @@
       <c r="X59" t="n">
         <v>0.007820000000000001</v>
       </c>
-      <c r="Y59" s="4" t="n">
+      <c r="Y59" t="n">
         <v>4</v>
       </c>
-      <c r="Z59" s="4" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="AA59" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="Z59" t="n">
+        <v>0.0587</v>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AC59" t="n">
@@ -6759,7 +6759,7 @@
         <v>4</v>
       </c>
       <c r="AE59" s="4" t="n">
-        <v>0.0321</v>
+        <v>0.0328</v>
       </c>
       <c r="AF59" s="4" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
         <v>7</v>
       </c>
       <c r="AJ59" t="n">
-        <v>0.155</v>
+        <v>0.17</v>
       </c>
       <c r="AK59" t="inlineStr">
         <is>
@@ -6858,7 +6858,7 @@
         <v>6</v>
       </c>
       <c r="Z60" t="n">
-        <v>0.328</v>
+        <v>0.447</v>
       </c>
       <c r="AA60" t="inlineStr">
         <is>
@@ -6872,7 +6872,7 @@
         <v>6</v>
       </c>
       <c r="AE60" t="n">
-        <v>0.37</v>
+        <v>0.404</v>
       </c>
       <c r="AF60" t="inlineStr">
         <is>
@@ -6886,7 +6886,7 @@
         <v>4</v>
       </c>
       <c r="AJ60" t="n">
-        <v>0.0946</v>
+        <v>0.1</v>
       </c>
       <c r="AK60" t="inlineStr">
         <is>
@@ -7084,7 +7084,7 @@
         <v>10</v>
       </c>
       <c r="Z62" t="n">
-        <v>0.446</v>
+        <v>0.608</v>
       </c>
       <c r="AA62" t="inlineStr">
         <is>
@@ -7112,7 +7112,7 @@
         <v>8</v>
       </c>
       <c r="AJ62" t="n">
-        <v>0.293</v>
+        <v>0.388</v>
       </c>
       <c r="AK62" t="inlineStr">
         <is>
@@ -7197,7 +7197,7 @@
         <v>8</v>
       </c>
       <c r="Z63" t="n">
-        <v>0.16</v>
+        <v>0.155</v>
       </c>
       <c r="AA63" t="inlineStr">
         <is>
@@ -7211,7 +7211,7 @@
         <v>8</v>
       </c>
       <c r="AE63" t="n">
-        <v>1</v>
+        <v>0.951</v>
       </c>
       <c r="AF63" t="inlineStr">
         <is>
@@ -7221,15 +7221,15 @@
       <c r="AH63" t="n">
         <v>0.0149</v>
       </c>
-      <c r="AI63" s="4" t="n">
+      <c r="AI63" t="n">
         <v>2</v>
       </c>
-      <c r="AJ63" s="4" t="n">
-        <v>0.0429</v>
-      </c>
-      <c r="AK63" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="AJ63" t="n">
+        <v>0.0585</v>
+      </c>
+      <c r="AK63" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -7310,7 +7310,7 @@
         <v>14</v>
       </c>
       <c r="Z64" t="n">
-        <v>0.669</v>
+        <v>0.651</v>
       </c>
       <c r="AA64" t="inlineStr">
         <is>
@@ -7324,7 +7324,7 @@
         <v>9</v>
       </c>
       <c r="AE64" t="n">
-        <v>0.705</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="AF64" t="inlineStr">
         <is>
@@ -7423,7 +7423,7 @@
         <v>9</v>
       </c>
       <c r="Z65" t="n">
-        <v>0.462</v>
+        <v>0.63</v>
       </c>
       <c r="AA65" t="inlineStr">
         <is>
@@ -7451,7 +7451,7 @@
         <v>3</v>
       </c>
       <c r="AJ65" t="n">
-        <v>0.138</v>
+        <v>0.09660000000000001</v>
       </c>
       <c r="AK65" t="inlineStr">
         <is>
@@ -7649,7 +7649,7 @@
         <v>7</v>
       </c>
       <c r="Z67" t="n">
-        <v>0.171</v>
+        <v>0.234</v>
       </c>
       <c r="AA67" t="inlineStr">
         <is>
@@ -7663,7 +7663,7 @@
         <v>5</v>
       </c>
       <c r="AE67" t="n">
-        <v>0.147</v>
+        <v>0.201</v>
       </c>
       <c r="AF67" t="inlineStr">
         <is>
@@ -7677,7 +7677,7 @@
         <v>9</v>
       </c>
       <c r="AJ67" t="n">
-        <v>0.492</v>
+        <v>0.509</v>
       </c>
       <c r="AK67" t="inlineStr">
         <is>
@@ -7762,7 +7762,7 @@
         <v>2</v>
       </c>
       <c r="Z68" s="3" t="n">
-        <v>2.23e-05</v>
+        <v>3.05e-05</v>
       </c>
       <c r="AA68" s="3" t="inlineStr">
         <is>
@@ -7776,7 +7776,7 @@
         <v>1</v>
       </c>
       <c r="AE68" s="3" t="n">
-        <v>0.00113</v>
+        <v>0.00154</v>
       </c>
       <c r="AF68" s="3" t="inlineStr">
         <is>
@@ -7790,7 +7790,7 @@
         <v>5</v>
       </c>
       <c r="AJ68" t="n">
-        <v>0.168</v>
+        <v>0.114</v>
       </c>
       <c r="AK68" t="inlineStr">
         <is>
@@ -7875,7 +7875,7 @@
         <v>1</v>
       </c>
       <c r="Z69" s="3" t="n">
-        <v>8.440000000000001e-06</v>
+        <v>1.15e-05</v>
       </c>
       <c r="AA69" s="3" t="inlineStr">
         <is>
@@ -7889,7 +7889,7 @@
         <v>2</v>
       </c>
       <c r="AE69" s="3" t="n">
-        <v>0.00426</v>
+        <v>0.0058</v>
       </c>
       <c r="AF69" s="3" t="inlineStr">
         <is>
@@ -7903,7 +7903,7 @@
         <v>6</v>
       </c>
       <c r="AJ69" t="n">
-        <v>0.216</v>
+        <v>0.218</v>
       </c>
       <c r="AK69" t="inlineStr">
         <is>
@@ -7990,7 +7990,7 @@
         <v>6</v>
       </c>
       <c r="Z72" t="n">
-        <v>0.389</v>
+        <v>0.477</v>
       </c>
       <c r="AA72" t="inlineStr">
         <is>
@@ -8004,7 +8004,7 @@
         <v>11</v>
       </c>
       <c r="AE72" t="n">
-        <v>0.983</v>
+        <v>0.928</v>
       </c>
       <c r="AF72" t="inlineStr">
         <is>
@@ -8103,7 +8103,7 @@
         <v>2</v>
       </c>
       <c r="Z73" t="n">
-        <v>0.0997</v>
+        <v>0.0906</v>
       </c>
       <c r="AA73" t="inlineStr">
         <is>
@@ -8117,7 +8117,7 @@
         <v>1</v>
       </c>
       <c r="AE73" s="4" t="n">
-        <v>0.0415</v>
+        <v>0.0396</v>
       </c>
       <c r="AF73" s="4" t="inlineStr">
         <is>
@@ -8131,7 +8131,7 @@
         <v>3</v>
       </c>
       <c r="AJ73" t="n">
-        <v>0.367</v>
+        <v>0.5</v>
       </c>
       <c r="AK73" t="inlineStr">
         <is>
@@ -8244,7 +8244,7 @@
         <v>7</v>
       </c>
       <c r="AJ74" t="n">
-        <v>0.752</v>
+        <v>1</v>
       </c>
       <c r="AK74" t="inlineStr">
         <is>
@@ -8329,7 +8329,7 @@
         <v>5</v>
       </c>
       <c r="Z75" t="n">
-        <v>0.381</v>
+        <v>0.519</v>
       </c>
       <c r="AA75" t="inlineStr">
         <is>
@@ -8357,7 +8357,7 @@
         <v>6</v>
       </c>
       <c r="AJ75" t="n">
-        <v>0.726</v>
+        <v>0.99</v>
       </c>
       <c r="AK75" t="inlineStr">
         <is>
@@ -8555,7 +8555,7 @@
         <v>8</v>
       </c>
       <c r="Z77" t="n">
-        <v>0.49</v>
+        <v>0.547</v>
       </c>
       <c r="AA77" t="inlineStr">
         <is>
@@ -8569,7 +8569,7 @@
         <v>5</v>
       </c>
       <c r="AE77" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="AF77" t="inlineStr">
         <is>
@@ -8583,7 +8583,7 @@
         <v>2</v>
       </c>
       <c r="AJ77" t="n">
-        <v>0.155</v>
+        <v>0.164</v>
       </c>
       <c r="AK77" t="inlineStr">
         <is>
@@ -8668,7 +8668,7 @@
         <v>9</v>
       </c>
       <c r="Z78" t="n">
-        <v>0.822</v>
+        <v>1</v>
       </c>
       <c r="AA78" t="inlineStr">
         <is>
@@ -8682,7 +8682,7 @@
         <v>8</v>
       </c>
       <c r="AE78" t="n">
-        <v>0.554</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="AF78" t="inlineStr">
         <is>
@@ -8696,7 +8696,7 @@
         <v>10</v>
       </c>
       <c r="AJ78" t="n">
-        <v>0.309</v>
+        <v>0.313</v>
       </c>
       <c r="AK78" t="inlineStr">
         <is>
@@ -8894,7 +8894,7 @@
         <v>7</v>
       </c>
       <c r="Z80" t="n">
-        <v>0.548</v>
+        <v>0.748</v>
       </c>
       <c r="AA80" t="inlineStr">
         <is>
@@ -8922,7 +8922,7 @@
         <v>11</v>
       </c>
       <c r="AJ80" t="n">
-        <v>0.401</v>
+        <v>0.478</v>
       </c>
       <c r="AK80" t="inlineStr">
         <is>
@@ -9007,7 +9007,7 @@
         <v>2</v>
       </c>
       <c r="Z81" t="n">
-        <v>0.16</v>
+        <v>0.155</v>
       </c>
       <c r="AA81" t="inlineStr">
         <is>
@@ -9021,7 +9021,7 @@
         <v>7</v>
       </c>
       <c r="AE81" t="n">
-        <v>0.748</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="AF81" t="inlineStr">
         <is>
@@ -9035,7 +9035,7 @@
         <v>4</v>
       </c>
       <c r="AJ81" t="n">
-        <v>0.187</v>
+        <v>0.255</v>
       </c>
       <c r="AK81" t="inlineStr">
         <is>
@@ -9120,7 +9120,7 @@
         <v>11</v>
       </c>
       <c r="Z82" t="n">
-        <v>0.669</v>
+        <v>0.651</v>
       </c>
       <c r="AA82" t="inlineStr">
         <is>
@@ -9134,7 +9134,7 @@
         <v>10</v>
       </c>
       <c r="AE82" t="n">
-        <v>0.702</v>
+        <v>0.662</v>
       </c>
       <c r="AF82" t="inlineStr">
         <is>
@@ -9148,7 +9148,7 @@
         <v>9</v>
       </c>
       <c r="AJ82" t="n">
-        <v>0.414</v>
+        <v>0.484</v>
       </c>
       <c r="AK82" t="inlineStr">
         <is>
@@ -9247,7 +9247,7 @@
         <v>9</v>
       </c>
       <c r="AE83" t="n">
-        <v>0.536</v>
+        <v>0.522</v>
       </c>
       <c r="AF83" t="inlineStr">
         <is>
@@ -9360,7 +9360,7 @@
         <v>6</v>
       </c>
       <c r="AE84" t="n">
-        <v>0.611</v>
+        <v>0.666</v>
       </c>
       <c r="AF84" t="inlineStr">
         <is>
@@ -9374,7 +9374,7 @@
         <v>1</v>
       </c>
       <c r="AJ84" t="n">
-        <v>0.369</v>
+        <v>0.503</v>
       </c>
       <c r="AK84" t="inlineStr">
         <is>
@@ -9459,7 +9459,7 @@
         <v>10</v>
       </c>
       <c r="Z85" t="n">
-        <v>0.708</v>
+        <v>0.864</v>
       </c>
       <c r="AA85" t="inlineStr">
         <is>
@@ -9473,7 +9473,7 @@
         <v>3</v>
       </c>
       <c r="AE85" t="n">
-        <v>0.16</v>
+        <v>0.219</v>
       </c>
       <c r="AF85" t="inlineStr">
         <is>
@@ -9487,7 +9487,7 @@
         <v>13</v>
       </c>
       <c r="AJ85" t="n">
-        <v>0.492</v>
+        <v>0.509</v>
       </c>
       <c r="AK85" t="inlineStr">
         <is>
@@ -9572,7 +9572,7 @@
         <v>4</v>
       </c>
       <c r="Z86" t="n">
-        <v>0.137</v>
+        <v>0.145</v>
       </c>
       <c r="AA86" t="inlineStr">
         <is>
@@ -9586,7 +9586,7 @@
         <v>2</v>
       </c>
       <c r="AE86" t="n">
-        <v>0.101</v>
+        <v>0.137</v>
       </c>
       <c r="AF86" t="inlineStr">
         <is>
@@ -9600,7 +9600,7 @@
         <v>8</v>
       </c>
       <c r="AJ86" t="n">
-        <v>0.301</v>
+        <v>0.274</v>
       </c>
       <c r="AK86" t="inlineStr">
         <is>
@@ -9681,15 +9681,15 @@
       <c r="X87" t="n">
         <v>0.0261</v>
       </c>
-      <c r="Y87" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z87" s="4" t="n">
-        <v>0.041</v>
-      </c>
-      <c r="AA87" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="Y87" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z87" t="n">
+        <v>0.0559</v>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AC87" t="n">
@@ -9699,7 +9699,7 @@
         <v>4</v>
       </c>
       <c r="AE87" t="n">
-        <v>0.176</v>
+        <v>0.24</v>
       </c>
       <c r="AF87" t="inlineStr">
         <is>
@@ -9713,7 +9713,7 @@
         <v>5</v>
       </c>
       <c r="AJ87" t="n">
-        <v>0.216</v>
+        <v>0.221</v>
       </c>
       <c r="AK87" t="inlineStr">
         <is>
@@ -9799,7 +9799,7 @@
         <v>6</v>
       </c>
       <c r="Z89" t="n">
-        <v>0.429</v>
+        <v>0.488</v>
       </c>
       <c r="AA89" t="inlineStr">
         <is>
@@ -9813,7 +9813,7 @@
         <v>1</v>
       </c>
       <c r="AE89" s="3" t="n">
-        <v>0.00152</v>
+        <v>0.00207</v>
       </c>
       <c r="AF89" s="3" t="inlineStr">
         <is>
@@ -9827,7 +9827,7 @@
         <v>1</v>
       </c>
       <c r="AJ89" s="3" t="n">
-        <v>3.33e-06</v>
+        <v>4.54e-06</v>
       </c>
       <c r="AK89" s="3" t="inlineStr">
         <is>
@@ -9912,7 +9912,7 @@
         <v>2</v>
       </c>
       <c r="Z90" s="4" t="n">
-        <v>0.0178</v>
+        <v>0.0154</v>
       </c>
       <c r="AA90" s="4" t="inlineStr">
         <is>
@@ -9926,7 +9926,7 @@
         <v>7</v>
       </c>
       <c r="AE90" t="n">
-        <v>0.161</v>
+        <v>0.146</v>
       </c>
       <c r="AF90" t="inlineStr">
         <is>
@@ -10039,7 +10039,7 @@
         <v>13</v>
       </c>
       <c r="AE91" t="n">
-        <v>0.91</v>
+        <v>0.886</v>
       </c>
       <c r="AF91" t="inlineStr">
         <is>
@@ -10053,7 +10053,7 @@
         <v>9</v>
       </c>
       <c r="AJ91" t="n">
-        <v>0.968</v>
+        <v>1</v>
       </c>
       <c r="AK91" t="inlineStr">
         <is>
@@ -10152,7 +10152,7 @@
         <v>8</v>
       </c>
       <c r="AE92" t="n">
-        <v>0.333</v>
+        <v>0.454</v>
       </c>
       <c r="AF92" t="inlineStr">
         <is>
@@ -10251,7 +10251,7 @@
         <v>7</v>
       </c>
       <c r="Z93" t="n">
-        <v>1</v>
+        <v>0.787</v>
       </c>
       <c r="AA93" t="inlineStr">
         <is>
@@ -10265,7 +10265,7 @@
         <v>6</v>
       </c>
       <c r="AE93" t="n">
-        <v>0.228</v>
+        <v>0.155</v>
       </c>
       <c r="AF93" t="inlineStr">
         <is>
@@ -10279,7 +10279,7 @@
         <v>7</v>
       </c>
       <c r="AJ93" t="n">
-        <v>0.12</v>
+        <v>0.164</v>
       </c>
       <c r="AK93" t="inlineStr">
         <is>
@@ -10364,7 +10364,7 @@
         <v>4</v>
       </c>
       <c r="Z94" t="n">
-        <v>0.169</v>
+        <v>0.23</v>
       </c>
       <c r="AA94" t="inlineStr">
         <is>
@@ -10378,7 +10378,7 @@
         <v>2</v>
       </c>
       <c r="AE94" s="4" t="n">
-        <v>0.0121</v>
+        <v>0.011</v>
       </c>
       <c r="AF94" s="4" t="inlineStr">
         <is>
@@ -10392,7 +10392,7 @@
         <v>3</v>
       </c>
       <c r="AJ94" s="3" t="n">
-        <v>0.000103</v>
+        <v>4.7e-05</v>
       </c>
       <c r="AK94" s="3" t="inlineStr">
         <is>
@@ -10477,7 +10477,7 @@
         <v>8</v>
       </c>
       <c r="Z95" t="n">
-        <v>0.822</v>
+        <v>1</v>
       </c>
       <c r="AA95" t="inlineStr">
         <is>
@@ -10491,7 +10491,7 @@
         <v>4</v>
       </c>
       <c r="AE95" t="n">
-        <v>0.08169999999999999</v>
+        <v>0.0742</v>
       </c>
       <c r="AF95" t="inlineStr">
         <is>
@@ -10505,7 +10505,7 @@
         <v>2</v>
       </c>
       <c r="AJ95" s="3" t="n">
-        <v>2.3e-05</v>
+        <v>3.13e-05</v>
       </c>
       <c r="AK95" s="3" t="inlineStr">
         <is>
@@ -10586,15 +10586,15 @@
       <c r="X96" t="n">
         <v>0.0131</v>
       </c>
-      <c r="Y96" s="4" t="n">
+      <c r="Y96" t="n">
         <v>3</v>
       </c>
-      <c r="Z96" s="4" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="AA96" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="Z96" t="n">
+        <v>0.0655</v>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AC96" t="n">
@@ -10604,7 +10604,7 @@
         <v>11</v>
       </c>
       <c r="AE96" t="n">
-        <v>0.951</v>
+        <v>0.945</v>
       </c>
       <c r="AF96" t="inlineStr">
         <is>
@@ -10703,7 +10703,7 @@
         <v>1</v>
       </c>
       <c r="Z97" s="4" t="n">
-        <v>0.0172</v>
+        <v>0.0234</v>
       </c>
       <c r="AA97" s="4" t="inlineStr">
         <is>
@@ -10717,7 +10717,7 @@
         <v>12</v>
       </c>
       <c r="AE97" t="n">
-        <v>0.913</v>
+        <v>0.9</v>
       </c>
       <c r="AF97" t="inlineStr">
         <is>
@@ -10731,7 +10731,7 @@
         <v>6</v>
       </c>
       <c r="AJ97" s="3" t="n">
-        <v>0.00091</v>
+        <v>0.00124</v>
       </c>
       <c r="AK97" s="3" t="inlineStr">
         <is>
@@ -10830,7 +10830,7 @@
         <v>10</v>
       </c>
       <c r="AE98" t="n">
-        <v>0.748</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="AF98" t="inlineStr">
         <is>
@@ -10844,7 +10844,7 @@
         <v>10</v>
       </c>
       <c r="AJ98" t="n">
-        <v>0.509</v>
+        <v>0.608</v>
       </c>
       <c r="AK98" t="inlineStr">
         <is>
@@ -10929,7 +10929,7 @@
         <v>5</v>
       </c>
       <c r="Z99" t="n">
-        <v>0.193</v>
+        <v>0.175</v>
       </c>
       <c r="AA99" t="inlineStr">
         <is>
@@ -10943,7 +10943,7 @@
         <v>3</v>
       </c>
       <c r="AE99" t="n">
-        <v>0.0737</v>
+        <v>0.0603</v>
       </c>
       <c r="AF99" t="inlineStr">
         <is>
@@ -11056,7 +11056,7 @@
         <v>5</v>
       </c>
       <c r="AE100" t="n">
-        <v>0.186</v>
+        <v>0.191</v>
       </c>
       <c r="AF100" t="inlineStr">
         <is>
@@ -11070,7 +11070,7 @@
         <v>4</v>
       </c>
       <c r="AJ100" s="3" t="n">
-        <v>0.000436</v>
+        <v>0.000198</v>
       </c>
       <c r="AK100" s="3" t="inlineStr">
         <is>
@@ -11268,7 +11268,7 @@
         <v>11</v>
       </c>
       <c r="Z102" t="n">
-        <v>0.76</v>
+        <v>0.864</v>
       </c>
       <c r="AA102" t="inlineStr">
         <is>
@@ -11282,7 +11282,7 @@
         <v>9</v>
       </c>
       <c r="AE102" t="n">
-        <v>0.19</v>
+        <v>0.259</v>
       </c>
       <c r="AF102" t="inlineStr">
         <is>
@@ -11296,7 +11296,7 @@
         <v>5</v>
       </c>
       <c r="AJ102" s="3" t="n">
-        <v>0.000812</v>
+        <v>0.00111</v>
       </c>
       <c r="AK102" s="3" t="inlineStr">
         <is>
@@ -11409,7 +11409,7 @@
         <v>8</v>
       </c>
       <c r="AJ103" t="n">
-        <v>0.363</v>
+        <v>0.354</v>
       </c>
       <c r="AK103" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
         <v>9</v>
       </c>
       <c r="Z104" t="n">
-        <v>0.708</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AA104" t="inlineStr">
         <is>
@@ -11508,7 +11508,7 @@
         <v>14</v>
       </c>
       <c r="AE104" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.987</v>
       </c>
       <c r="AF104" t="inlineStr">
         <is>
@@ -15648,7 +15648,7 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.000462</v>
+        <v>0.000472</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -15662,7 +15662,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>0.000341</v>
+        <v>0.00031</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -15676,7 +15676,7 @@
         <v>8</v>
       </c>
       <c r="X2" t="n">
-        <v>0.294</v>
+        <v>0.302</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
@@ -15713,7 +15713,7 @@
         <v>8</v>
       </c>
       <c r="I3" t="n">
-        <v>0.739</v>
+        <v>0.742</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -15727,7 +15727,7 @@
         <v>4</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0429</v>
+        <v>0.0472</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -15741,7 +15741,7 @@
         <v>2</v>
       </c>
       <c r="S3" t="n">
-        <v>0.00277</v>
+        <v>0.00309</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -15755,7 +15755,7 @@
         <v>5</v>
       </c>
       <c r="X3" t="n">
-        <v>0.131</v>
+        <v>0.139</v>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
@@ -15792,7 +15792,7 @@
         <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0295</v>
+        <v>0.0342</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -15806,7 +15806,7 @@
         <v>2</v>
       </c>
       <c r="N4" t="n">
-        <v>0.00396</v>
+        <v>0.00415</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -15820,7 +15820,7 @@
         <v>7</v>
       </c>
       <c r="S4" t="n">
-        <v>0.157</v>
+        <v>0.165</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -15834,7 +15834,7 @@
         <v>4</v>
       </c>
       <c r="X4" t="n">
-        <v>0.0295</v>
+        <v>0.0342</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
@@ -15871,7 +15871,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>0.004</v>
+        <v>0.00429</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -15885,7 +15885,7 @@
         <v>7</v>
       </c>
       <c r="N5" t="n">
-        <v>0.138</v>
+        <v>0.144</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -15899,7 +15899,7 @@
         <v>4</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0242</v>
+        <v>0.0275</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -15913,7 +15913,7 @@
         <v>2</v>
       </c>
       <c r="X5" t="n">
-        <v>0.0105</v>
+        <v>0.0118</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
@@ -15950,7 +15950,7 @@
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0151</v>
+        <v>0.0172</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -15964,7 +15964,7 @@
         <v>6</v>
       </c>
       <c r="N6" t="n">
-        <v>0.0868</v>
+        <v>0.0905</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -15978,7 +15978,7 @@
         <v>3</v>
       </c>
       <c r="S6" t="n">
-        <v>0.008659999999999999</v>
+        <v>0.009480000000000001</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -15992,7 +15992,7 @@
         <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>0.008659999999999999</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
@@ -16029,7 +16029,7 @@
         <v>6</v>
       </c>
       <c r="I7" t="n">
-        <v>0.221</v>
+        <v>0.23</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -16043,7 +16043,7 @@
         <v>3</v>
       </c>
       <c r="N7" t="n">
-        <v>0.0198</v>
+        <v>0.0228</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -16057,7 +16057,7 @@
         <v>5</v>
       </c>
       <c r="S7" t="n">
-        <v>0.026</v>
+        <v>0.0298</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -16071,7 +16071,7 @@
         <v>6</v>
       </c>
       <c r="X7" t="n">
-        <v>0.159</v>
+        <v>0.168</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -16108,7 +16108,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>0.023</v>
+        <v>0.0269</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -16122,7 +16122,7 @@
         <v>8</v>
       </c>
       <c r="N8" t="n">
-        <v>0.214</v>
+        <v>0.22</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -16136,7 +16136,7 @@
         <v>6</v>
       </c>
       <c r="S8" t="n">
-        <v>0.0945</v>
+        <v>0.0994</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -16150,7 +16150,7 @@
         <v>3</v>
       </c>
       <c r="X8" t="n">
-        <v>0.0211</v>
+        <v>0.0245</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -16187,7 +16187,7 @@
         <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0242</v>
+        <v>0.0274</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -16201,7 +16201,7 @@
         <v>9</v>
       </c>
       <c r="N9" t="n">
-        <v>0.821</v>
+        <v>0.83</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -16215,7 +16215,7 @@
         <v>8</v>
       </c>
       <c r="S9" t="n">
-        <v>0.164</v>
+        <v>0.174</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -16229,7 +16229,7 @@
         <v>7</v>
       </c>
       <c r="X9" t="n">
-        <v>0.251</v>
+        <v>0.262</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -16266,7 +16266,7 @@
         <v>7</v>
       </c>
       <c r="I10" t="n">
-        <v>0.425</v>
+        <v>0.445</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -16280,7 +16280,7 @@
         <v>5</v>
       </c>
       <c r="N10" t="n">
-        <v>0.0429</v>
+        <v>0.0472</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -16294,7 +16294,7 @@
         <v>9</v>
       </c>
       <c r="S10" t="n">
-        <v>0.303</v>
+        <v>0.314</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -16308,7 +16308,7 @@
         <v>9</v>
       </c>
       <c r="X10" t="n">
-        <v>0.537</v>
+        <v>0.556</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -16346,7 +16346,7 @@
         <v>9</v>
       </c>
       <c r="I12" t="n">
-        <v>0.839</v>
+        <v>0.834</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -16360,7 +16360,7 @@
         <v>1</v>
       </c>
       <c r="N12" t="n">
-        <v>0.00135</v>
+        <v>0.00115</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -16374,7 +16374,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>0.000671</v>
+        <v>0.00061</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
@@ -16388,7 +16388,7 @@
         <v>8</v>
       </c>
       <c r="X12" t="n">
-        <v>0.263</v>
+        <v>0.269</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
@@ -16425,7 +16425,7 @@
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>0.00636</v>
+        <v>0.00705</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -16439,7 +16439,7 @@
         <v>2</v>
       </c>
       <c r="N13" t="n">
-        <v>0.00483</v>
+        <v>0.00494</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -16453,7 +16453,7 @@
         <v>8</v>
       </c>
       <c r="S13" t="n">
-        <v>0.193</v>
+        <v>0.195</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -16467,7 +16467,7 @@
         <v>4</v>
       </c>
       <c r="X13" t="n">
-        <v>0.0176</v>
+        <v>0.0207</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         <v>4</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0212</v>
+        <v>0.0254</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -16518,7 +16518,7 @@
         <v>6</v>
       </c>
       <c r="N14" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.08260000000000001</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -16532,7 +16532,7 @@
         <v>3</v>
       </c>
       <c r="S14" t="n">
-        <v>0.014</v>
+        <v>0.0162</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -16546,7 +16546,7 @@
         <v>1</v>
       </c>
       <c r="X14" t="n">
-        <v>0.00532</v>
+        <v>0.00558</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
@@ -16583,7 +16583,7 @@
         <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>0.00584</v>
+        <v>0.00626</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -16597,7 +16597,7 @@
         <v>8</v>
       </c>
       <c r="N15" t="n">
-        <v>0.263</v>
+        <v>0.271</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -16611,7 +16611,7 @@
         <v>5</v>
       </c>
       <c r="S15" t="n">
-        <v>0.0253</v>
+        <v>0.0273</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -16625,7 +16625,7 @@
         <v>2</v>
       </c>
       <c r="X15" t="n">
-        <v>0.00899</v>
+        <v>0.0101</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
@@ -16662,7 +16662,7 @@
         <v>7</v>
       </c>
       <c r="I16" t="n">
-        <v>0.465</v>
+        <v>0.479</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -16676,7 +16676,7 @@
         <v>3</v>
       </c>
       <c r="N16" t="n">
-        <v>0.00636</v>
+        <v>0.00705</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -16690,7 +16690,7 @@
         <v>4</v>
       </c>
       <c r="S16" t="n">
-        <v>0.0188</v>
+        <v>0.0225</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
@@ -16704,7 +16704,7 @@
         <v>7</v>
       </c>
       <c r="X16" t="n">
-        <v>0.206</v>
+        <v>0.212</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
@@ -16741,7 +16741,7 @@
         <v>6</v>
       </c>
       <c r="I17" t="n">
-        <v>0.393</v>
+        <v>0.402</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -16755,7 +16755,7 @@
         <v>4</v>
       </c>
       <c r="N17" t="n">
-        <v>0.009860000000000001</v>
+        <v>0.0112</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -16769,7 +16769,7 @@
         <v>9</v>
       </c>
       <c r="S17" t="n">
-        <v>0.263</v>
+        <v>0.271</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
@@ -16820,7 +16820,7 @@
         <v>8</v>
       </c>
       <c r="I18" t="n">
-        <v>0.839</v>
+        <v>0.829</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -16834,7 +16834,7 @@
         <v>5</v>
       </c>
       <c r="N18" t="n">
-        <v>0.06270000000000001</v>
+        <v>0.0668</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -16848,7 +16848,7 @@
         <v>2</v>
       </c>
       <c r="S18" t="n">
-        <v>0.0104</v>
+        <v>0.0119</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -16862,7 +16862,7 @@
         <v>6</v>
       </c>
       <c r="X18" t="n">
-        <v>0.154</v>
+        <v>0.162</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
@@ -16899,7 +16899,7 @@
         <v>3</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0188</v>
+        <v>0.0225</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -16913,7 +16913,7 @@
         <v>7</v>
       </c>
       <c r="N19" t="n">
-        <v>0.105</v>
+        <v>0.112</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -16927,7 +16927,7 @@
         <v>6</v>
       </c>
       <c r="S19" t="n">
-        <v>0.09039999999999999</v>
+        <v>0.0951</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
@@ -16941,7 +16941,7 @@
         <v>3</v>
       </c>
       <c r="X19" t="n">
-        <v>0.0154</v>
+        <v>0.018</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
@@ -16978,7 +16978,7 @@
         <v>5</v>
       </c>
       <c r="I20" t="n">
-        <v>0.0445</v>
+        <v>0.0486</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -16992,7 +16992,7 @@
         <v>9</v>
       </c>
       <c r="N20" t="n">
-        <v>0.494</v>
+        <v>0.504</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -17006,7 +17006,7 @@
         <v>7</v>
       </c>
       <c r="S20" t="n">
-        <v>0.159</v>
+        <v>0.164</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
@@ -17020,7 +17020,7 @@
         <v>5</v>
       </c>
       <c r="X20" t="n">
-        <v>0.103</v>
+        <v>0.109</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
reorganize rag outputs and refresh figures
</commit_message>
<xml_diff>
--- a/rag/eval/results_full150/SuppFile2_Stats_generated.xlsx
+++ b/rag/eval/results_full150/SuppFile2_Stats_generated.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="IndividQuest_FisherExact(Tab3)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ModelComp_SignedRankFig4" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ModelComp_BH_AdjustFig4" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IndividQuest_FisherExact(Tab3)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelComp_SignedRankFig4" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelComp_BH_AdjustFig4" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1695,10 +1695,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F11" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G11" t="n">
         <v>5</v>
@@ -1707,16 +1707,16 @@
         <v>64</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.9275</v>
+        <v>0.9286</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0.7901</v>
+        <v>0.8025</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.8609</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1724,10 +1724,10 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q11" t="n">
         <v>5</v>
@@ -1736,25 +1736,25 @@
         <v>64</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>0.8733</v>
+        <v>0.88</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>0.9306</v>
+        <v>0.9315</v>
       </c>
       <c r="U11" s="2" t="n">
-        <v>0.8272</v>
+        <v>0.8395</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>0.8758</v>
+        <v>0.8831</v>
       </c>
       <c r="X11" t="n">
-        <v>0.737</v>
+        <v>0.732</v>
       </c>
       <c r="Y11" t="n">
         <v>11</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.85</v>
+        <v>0.949</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -1776,13 +1776,13 @@
         </is>
       </c>
       <c r="AH11" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="AI11" t="n">
         <v>11</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.862</v>
+        <v>0.858</v>
       </c>
       <c r="AK11" t="inlineStr">
         <is>
@@ -2897,7 +2897,7 @@
         <v>1</v>
       </c>
       <c r="Y22" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z22" t="n">
         <v>1</v>
@@ -3010,7 +3010,7 @@
         <v>1</v>
       </c>
       <c r="Y23" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z23" t="n">
         <v>1</v>
@@ -3519,10 +3519,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F28" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G28" t="n">
         <v>5</v>
@@ -3531,16 +3531,16 @@
         <v>64</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.9275</v>
+        <v>0.9286</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0.7901</v>
+        <v>0.8025</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.8609</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -3572,13 +3572,13 @@
         <v>0.8649</v>
       </c>
       <c r="X28" t="n">
-        <v>0.868</v>
+        <v>1</v>
       </c>
       <c r="Y28" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Z28" t="n">
-        <v>0.879</v>
+        <v>1</v>
       </c>
       <c r="AA28" t="inlineStr">
         <is>
@@ -3586,13 +3586,13 @@
         </is>
       </c>
       <c r="AC28" t="n">
-        <v>0.718</v>
+        <v>0.719</v>
       </c>
       <c r="AD28" t="n">
         <v>13</v>
       </c>
       <c r="AE28" t="n">
-        <v>0.979</v>
+        <v>0.98</v>
       </c>
       <c r="AF28" t="inlineStr">
         <is>
@@ -4027,7 +4027,7 @@
         <v>1</v>
       </c>
       <c r="Y32" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z32" t="n">
         <v>1</v>
@@ -4253,7 +4253,7 @@
         <v>1</v>
       </c>
       <c r="Y34" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z34" t="n">
         <v>1</v>
@@ -10050,7 +10050,7 @@
         <v>0.352</v>
       </c>
       <c r="AI91" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AJ91" t="n">
         <v>1</v>
@@ -10786,10 +10786,10 @@
         </is>
       </c>
       <c r="O98" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="P98" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q98" t="n">
         <v>7</v>
@@ -10798,25 +10798,25 @@
         <v>62</v>
       </c>
       <c r="S98" s="2" t="n">
-        <v>0.8333</v>
+        <v>0.84</v>
       </c>
       <c r="T98" s="2" t="n">
-        <v>0.9</v>
+        <v>0.9014</v>
       </c>
       <c r="U98" s="2" t="n">
-        <v>0.7778</v>
+        <v>0.7901</v>
       </c>
       <c r="V98" s="2" t="n">
-        <v>0.8344</v>
+        <v>0.8421</v>
       </c>
       <c r="X98" t="n">
-        <v>0.879</v>
+        <v>0.759</v>
       </c>
       <c r="Y98" t="n">
         <v>12</v>
       </c>
       <c r="Z98" t="n">
-        <v>0.879</v>
+        <v>0.949</v>
       </c>
       <c r="AA98" t="inlineStr">
         <is>
@@ -10824,13 +10824,13 @@
         </is>
       </c>
       <c r="AC98" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="AD98" t="n">
         <v>10</v>
       </c>
       <c r="AE98" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.572</v>
       </c>
       <c r="AF98" t="inlineStr">
         <is>
@@ -10838,13 +10838,13 @@
         </is>
       </c>
       <c r="AH98" t="n">
-        <v>0.37</v>
+        <v>0.278</v>
       </c>
       <c r="AI98" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AJ98" t="n">
-        <v>0.608</v>
+        <v>0.596</v>
       </c>
       <c r="AK98" t="inlineStr">
         <is>
@@ -11406,7 +11406,7 @@
         <v>0.33</v>
       </c>
       <c r="AI103" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AJ103" t="n">
         <v>0.354</v>
@@ -12110,7 +12110,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0.7867</v>
@@ -12122,7 +12122,7 @@
         <v>10</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0.9275</v>
+        <v>0.9286</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>0.9804</v>
@@ -12134,7 +12134,7 @@
         <v>10</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>0.7901</v>
+        <v>0.8025</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>0.6173</v>
@@ -12146,7 +12146,7 @@
         <v>10</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.8609</v>
       </c>
       <c r="S12" s="6" t="n">
         <v>0.7576000000000001</v>
@@ -13001,7 +13001,7 @@
         <v>10</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>0.8733</v>
+        <v>0.88</v>
       </c>
       <c r="D32" s="6" t="n">
         <v>0.8532999999999999</v>
@@ -13013,7 +13013,7 @@
         <v>10</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.9306</v>
+        <v>0.9315</v>
       </c>
       <c r="I32" s="6" t="n">
         <v>0.9683</v>
@@ -13025,7 +13025,7 @@
         <v>10</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.8272</v>
+        <v>0.8395</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>0.7531</v>
@@ -13037,7 +13037,7 @@
         <v>10</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>0.8758</v>
+        <v>0.8831</v>
       </c>
       <c r="S32" s="6" t="n">
         <v>0.8472</v>
@@ -13395,7 +13395,7 @@
         </is>
       </c>
       <c r="R39" t="n">
-        <v>0.00335</v>
+        <v>0.00336</v>
       </c>
       <c r="S39" t="n">
         <v>0.0154</v>
@@ -14014,7 +14014,7 @@
         <v>0.8733</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>0.8333</v>
+        <v>0.84</v>
       </c>
       <c r="G54" t="n">
         <v>10</v>
@@ -14026,7 +14026,7 @@
         <v>0.9559</v>
       </c>
       <c r="J54" s="6" t="n">
-        <v>0.9</v>
+        <v>0.9014</v>
       </c>
       <c r="L54" t="n">
         <v>10</v>
@@ -14038,7 +14038,7 @@
         <v>0.8025</v>
       </c>
       <c r="O54" s="6" t="n">
-        <v>0.7778</v>
+        <v>0.7901</v>
       </c>
       <c r="Q54" t="n">
         <v>10</v>
@@ -14050,7 +14050,7 @@
         <v>0.8725000000000001</v>
       </c>
       <c r="T54" s="6" t="n">
-        <v>0.8344</v>
+        <v>0.8421</v>
       </c>
     </row>
     <row r="55">
@@ -14360,13 +14360,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0.386</v>
+        <v>0.412</v>
       </c>
       <c r="D61" t="n">
         <v>0.0094</v>
       </c>
       <c r="E61" t="n">
-        <v>0.947</v>
+        <v>0.93</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -14374,13 +14374,13 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>0.0244</v>
+        <v>0.0242</v>
       </c>
       <c r="I61" t="n">
         <v>0.165</v>
       </c>
       <c r="J61" t="n">
-        <v>5.71e-05</v>
+        <v>5.82e-05</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -14388,13 +14388,13 @@
         </is>
       </c>
       <c r="M61" t="n">
-        <v>0.262</v>
+        <v>0.273</v>
       </c>
       <c r="N61" t="n">
         <v>0.058</v>
       </c>
       <c r="O61" t="n">
-        <v>3.1e-05</v>
+        <v>2.77e-05</v>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
@@ -14402,13 +14402,13 @@
         </is>
       </c>
       <c r="R61" t="n">
-        <v>0.5</v>
+        <v>0.487</v>
       </c>
       <c r="S61" t="n">
         <v>0.008160000000000001</v>
       </c>
       <c r="T61" t="n">
-        <v>0.247</v>
+        <v>0.238</v>
       </c>
     </row>
     <row r="62">
@@ -14418,7 +14418,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0.348</v>
+        <v>0.362</v>
       </c>
       <c r="D62" t="n">
         <v>0.008920000000000001</v>
@@ -14446,7 +14446,7 @@
         </is>
       </c>
       <c r="M62" t="n">
-        <v>0.221</v>
+        <v>0.198</v>
       </c>
       <c r="N62" t="n">
         <v>0.0555</v>
@@ -15367,7 +15367,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>0.0105</v>
+        <v>0.0112</v>
       </c>
       <c r="D83" t="n">
         <v>0.176</v>
@@ -15381,7 +15381,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>0.802</v>
+        <v>0.8</v>
       </c>
       <c r="I83" t="n">
         <v>0.00721</v>
@@ -15395,7 +15395,7 @@
         </is>
       </c>
       <c r="M83" t="n">
-        <v>0.119</v>
+        <v>0.124</v>
       </c>
       <c r="N83" t="n">
         <v>0.0124</v>
@@ -15409,7 +15409,7 @@
         </is>
       </c>
       <c r="R83" t="n">
-        <v>0.205</v>
+        <v>0.211</v>
       </c>
       <c r="S83" t="n">
         <v>0.112</v>
@@ -15425,7 +15425,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0.0243</v>
+        <v>0.0259</v>
       </c>
       <c r="D84" t="n">
         <v>0.423</v>
@@ -15628,13 +15628,13 @@
         <v>0.05</v>
       </c>
       <c r="G2" t="n">
-        <v>0.947</v>
+        <v>0.93</v>
       </c>
       <c r="H2" t="n">
         <v>9</v>
       </c>
       <c r="I2" t="n">
-        <v>0.947</v>
+        <v>0.93</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -15642,13 +15642,13 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>5.71e-05</v>
+        <v>5.82e-05</v>
       </c>
       <c r="M2" t="n">
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.000472</v>
+        <v>0.000466</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -15656,13 +15656,13 @@
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>3.1e-05</v>
+        <v>2.77e-05</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>0.00031</v>
+        <v>0.000277</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -15670,13 +15670,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>0.247</v>
+        <v>0.238</v>
       </c>
       <c r="W2" t="n">
         <v>8</v>
       </c>
       <c r="X2" t="n">
-        <v>0.302</v>
+        <v>0.286</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
@@ -15724,10 +15724,10 @@
         <v>0.0243</v>
       </c>
       <c r="M3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0472</v>
+        <v>0.047</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -15820,7 +15820,7 @@
         <v>7</v>
       </c>
       <c r="S4" t="n">
-        <v>0.165</v>
+        <v>0.168</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -15885,7 +15885,7 @@
         <v>7</v>
       </c>
       <c r="N5" t="n">
-        <v>0.144</v>
+        <v>0.148</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -15899,7 +15899,7 @@
         <v>4</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -15907,13 +15907,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.00335</v>
+        <v>0.00336</v>
       </c>
       <c r="W5" t="n">
         <v>2</v>
       </c>
       <c r="X5" t="n">
-        <v>0.0118</v>
+        <v>0.0119</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
@@ -16029,7 +16029,7 @@
         <v>6</v>
       </c>
       <c r="I7" t="n">
-        <v>0.23</v>
+        <v>0.235</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -16108,7 +16108,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0269</v>
+        <v>0.0256</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -16122,7 +16122,7 @@
         <v>8</v>
       </c>
       <c r="N8" t="n">
-        <v>0.22</v>
+        <v>0.225</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -16150,7 +16150,7 @@
         <v>3</v>
       </c>
       <c r="X8" t="n">
-        <v>0.0245</v>
+        <v>0.0233</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -16181,13 +16181,13 @@
         <v>0.05</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0105</v>
+        <v>0.0112</v>
       </c>
       <c r="H9" t="n">
         <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0274</v>
+        <v>0.028</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -16195,13 +16195,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0.802</v>
+        <v>0.8</v>
       </c>
       <c r="M9" t="n">
         <v>9</v>
       </c>
       <c r="N9" t="n">
-        <v>0.83</v>
+        <v>0.828</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -16209,13 +16209,13 @@
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>0.119</v>
+        <v>0.124</v>
       </c>
       <c r="R9" t="n">
         <v>8</v>
       </c>
       <c r="S9" t="n">
-        <v>0.174</v>
+        <v>0.181</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -16223,13 +16223,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.205</v>
+        <v>0.211</v>
       </c>
       <c r="W9" t="n">
         <v>7</v>
       </c>
       <c r="X9" t="n">
-        <v>0.262</v>
+        <v>0.269</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -16260,13 +16260,13 @@
         <v>0.05</v>
       </c>
       <c r="G10" t="n">
-        <v>0.386</v>
+        <v>0.412</v>
       </c>
       <c r="H10" t="n">
         <v>7</v>
       </c>
       <c r="I10" t="n">
-        <v>0.445</v>
+        <v>0.475</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -16274,13 +16274,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.0244</v>
+        <v>0.0242</v>
       </c>
       <c r="M10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" t="n">
-        <v>0.0472</v>
+        <v>0.047</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -16288,13 +16288,13 @@
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>0.262</v>
+        <v>0.273</v>
       </c>
       <c r="R10" t="n">
         <v>9</v>
       </c>
       <c r="S10" t="n">
-        <v>0.314</v>
+        <v>0.321</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -16302,13 +16302,13 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>0.5</v>
+        <v>0.487</v>
       </c>
       <c r="W10" t="n">
         <v>9</v>
       </c>
       <c r="X10" t="n">
-        <v>0.556</v>
+        <v>0.551</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         <v>4</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0254</v>
+        <v>0.0245</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -16597,7 +16597,7 @@
         <v>8</v>
       </c>
       <c r="N15" t="n">
-        <v>0.271</v>
+        <v>0.276</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -16611,7 +16611,7 @@
         <v>5</v>
       </c>
       <c r="S15" t="n">
-        <v>0.0273</v>
+        <v>0.0283</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -16662,7 +16662,7 @@
         <v>7</v>
       </c>
       <c r="I16" t="n">
-        <v>0.479</v>
+        <v>0.47</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -16690,7 +16690,7 @@
         <v>4</v>
       </c>
       <c r="S16" t="n">
-        <v>0.0225</v>
+        <v>0.0216</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
@@ -16735,13 +16735,13 @@
         <v>0.05</v>
       </c>
       <c r="G17" t="n">
-        <v>0.348</v>
+        <v>0.362</v>
       </c>
       <c r="H17" t="n">
         <v>6</v>
       </c>
       <c r="I17" t="n">
-        <v>0.402</v>
+        <v>0.418</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -16763,13 +16763,13 @@
         </is>
       </c>
       <c r="Q17" t="n">
-        <v>0.221</v>
+        <v>0.198</v>
       </c>
       <c r="R17" t="n">
         <v>9</v>
       </c>
       <c r="S17" t="n">
-        <v>0.271</v>
+        <v>0.258</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
@@ -16834,7 +16834,7 @@
         <v>5</v>
       </c>
       <c r="N18" t="n">
-        <v>0.0668</v>
+        <v>0.06469999999999999</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -16899,7 +16899,7 @@
         <v>3</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0225</v>
+        <v>0.0216</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -16972,17 +16972,17 @@
         <v>0.05</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0243</v>
+        <v>0.0259</v>
       </c>
       <c r="H20" t="n">
         <v>5</v>
       </c>
       <c r="I20" t="n">
-        <v>0.0486</v>
+        <v>0.0518</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -16992,7 +16992,7 @@
         <v>9</v>
       </c>
       <c r="N20" t="n">
-        <v>0.504</v>
+        <v>0.493</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -17006,7 +17006,7 @@
         <v>7</v>
       </c>
       <c r="S20" t="n">
-        <v>0.164</v>
+        <v>0.168</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Annotate lower-performing RAG significance results
Allow base comparison p-value annotations when intervention performance is worse than baseline, and regenerate RAG full150 figures and statistical summaries.
</commit_message>
<xml_diff>
--- a/rag/eval/results_full150/SuppFile2_Stats_generated.xlsx
+++ b/rag/eval/results_full150/SuppFile2_Stats_generated.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IndividQuest_FisherExact(Tab3)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelComp_SignedRankFig4" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelComp_BH_AdjustFig4" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="IndividQuest_FisherExact(Tab3)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ModelComp_SignedRankFig4" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ModelComp_BH_AdjustFig4" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>